<commit_message>
corr(data/ROL;TRO,IW): .xlsx + categorization_x.json
</commit_message>
<xml_diff>
--- a/data/Iwein/Iwein_final.xlsx
+++ b/data/Iwein/Iwein_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studsbgacat-my.sharepoint.com/personal/linda_beutel_studsbgacat_onmicrosoft_com/Documents/Studium/Dissertation/Programm/data/Iwein/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="11_2745FF4D7818D8D4D98E13AA110F1A3DC8184401" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3ABE7E17-8201-4208-AF10-B3DB88F36343}"/>
+  <xr:revisionPtr revIDLastSave="193" documentId="11_2745FF4D7818D8D4D98E13AA110F1A3DC8184401" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EFEC6658-28F0-42FB-9D77-090858ABE682}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="786" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="786" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gesamt" sheetId="1" r:id="rId1"/>
@@ -8166,7 +8166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -8184,21 +8184,20 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -9122,7 +9121,7 @@
       <c r="B17" s="9">
         <v>88</v>
       </c>
-      <c r="D17" s="13"/>
+      <c r="D17"/>
       <c r="F17" s="9" t="s">
         <v>43</v>
       </c>
@@ -9151,7 +9150,7 @@
       <c r="B19" s="9">
         <v>90</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="13" t="s">
         <v>35</v>
       </c>
       <c r="G19" s="9" t="s">
@@ -16423,7 +16422,7 @@
       </c>
     </row>
     <row r="446" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A446" s="15" t="s">
+      <c r="A446" s="14" t="s">
         <v>273</v>
       </c>
       <c r="B446" s="9">
@@ -16434,7 +16433,7 @@
       </c>
     </row>
     <row r="447" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A447" s="15" t="s">
+      <c r="A447" s="14" t="s">
         <v>21</v>
       </c>
       <c r="B447" s="9">
@@ -16556,7 +16555,7 @@
       </c>
     </row>
     <row r="454" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A454" s="15" t="s">
+      <c r="A454" s="14" t="s">
         <v>817</v>
       </c>
       <c r="B454" s="9">
@@ -17984,7 +17983,7 @@
       </c>
     </row>
     <row r="540" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A540" s="15" t="s">
+      <c r="A540" s="14" t="s">
         <v>21</v>
       </c>
       <c r="B540" s="9">
@@ -19328,7 +19327,7 @@
       <c r="E615" s="9" t="s">
         <v>1113</v>
       </c>
-      <c r="G615" s="16" t="s">
+      <c r="G615" s="15" t="s">
         <v>1114</v>
       </c>
       <c r="H615" s="10" t="s">
@@ -19348,7 +19347,7 @@
       <c r="E616" s="9" t="s">
         <v>590</v>
       </c>
-      <c r="G616" s="16" t="s">
+      <c r="G616" s="15" t="s">
         <v>1116</v>
       </c>
     </row>
@@ -19399,7 +19398,7 @@
       <c r="E619" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="G619" s="16" t="s">
+      <c r="G619" s="15" t="s">
         <v>1119</v>
       </c>
       <c r="H619" s="10" t="s">
@@ -19433,7 +19432,7 @@
       <c r="E621" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G621" s="16" t="s">
+      <c r="G621" s="15" t="s">
         <v>1121</v>
       </c>
       <c r="H621" s="10" t="s">
@@ -19470,7 +19469,7 @@
       <c r="E623" s="9" t="s">
         <v>1125</v>
       </c>
-      <c r="G623" s="16" t="s">
+      <c r="G623" s="15" t="s">
         <v>1126</v>
       </c>
       <c r="H623" s="10" t="s">
@@ -19490,7 +19489,7 @@
       <c r="E624" s="9" t="s">
         <v>1128</v>
       </c>
-      <c r="G624" s="16" t="s">
+      <c r="G624" s="15" t="s">
         <v>1129</v>
       </c>
     </row>
@@ -19507,7 +19506,7 @@
       <c r="E625" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G625" s="16" t="s">
+      <c r="G625" s="15" t="s">
         <v>1130</v>
       </c>
       <c r="H625" s="10" t="s">
@@ -19544,7 +19543,7 @@
       <c r="E627" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="G627" s="16" t="s">
+      <c r="G627" s="15" t="s">
         <v>1133</v>
       </c>
       <c r="H627" s="10" t="s">
@@ -19564,7 +19563,7 @@
       <c r="E628" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G628" s="16" t="s">
+      <c r="G628" s="15" t="s">
         <v>1135</v>
       </c>
     </row>
@@ -19581,7 +19580,7 @@
       <c r="E629" s="9" t="s">
         <v>1137</v>
       </c>
-      <c r="G629" s="16" t="s">
+      <c r="G629" s="15" t="s">
         <v>1138</v>
       </c>
     </row>
@@ -19635,7 +19634,7 @@
       <c r="E632" s="9" t="s">
         <v>1146</v>
       </c>
-      <c r="G632" s="16" t="s">
+      <c r="G632" s="15" t="s">
         <v>1147</v>
       </c>
     </row>
@@ -19669,7 +19668,7 @@
       <c r="E634" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="G634" s="16" t="s">
+      <c r="G634" s="15" t="s">
         <v>1148</v>
       </c>
       <c r="H634" s="10" t="s">
@@ -19689,7 +19688,7 @@
       <c r="E635" s="9" t="s">
         <v>1150</v>
       </c>
-      <c r="G635" s="16" t="s">
+      <c r="G635" s="15" t="s">
         <v>1151</v>
       </c>
     </row>
@@ -19706,7 +19705,7 @@
       <c r="E636" s="9" t="s">
         <v>705</v>
       </c>
-      <c r="G636" s="16" t="s">
+      <c r="G636" s="15" t="s">
         <v>1152</v>
       </c>
     </row>
@@ -19743,7 +19742,7 @@
       <c r="E638" s="9" t="s">
         <v>1156</v>
       </c>
-      <c r="G638" s="16" t="s">
+      <c r="G638" s="15" t="s">
         <v>1157</v>
       </c>
     </row>
@@ -19757,7 +19756,7 @@
       <c r="F639" s="9" t="s">
         <v>1158</v>
       </c>
-      <c r="G639" s="16" t="s">
+      <c r="G639" s="15" t="s">
         <v>1159</v>
       </c>
       <c r="H639" s="10" t="s">
@@ -19777,7 +19776,7 @@
       <c r="E640" s="9" t="s">
         <v>1161</v>
       </c>
-      <c r="G640" s="16" t="s">
+      <c r="G640" s="15" t="s">
         <v>1162</v>
       </c>
       <c r="H640" s="10" t="s">
@@ -19797,7 +19796,7 @@
       <c r="E641" s="9" t="s">
         <v>1164</v>
       </c>
-      <c r="G641" s="16" t="s">
+      <c r="G641" s="15" t="s">
         <v>1165</v>
       </c>
       <c r="H641" s="10" t="s">
@@ -19817,7 +19816,7 @@
       <c r="E642" s="9" t="s">
         <v>1167</v>
       </c>
-      <c r="G642" s="16" t="s">
+      <c r="G642" s="15" t="s">
         <v>1168</v>
       </c>
       <c r="H642" s="10" t="s">
@@ -19837,7 +19836,7 @@
       <c r="E643" s="9" t="s">
         <v>1170</v>
       </c>
-      <c r="G643" s="16" t="s">
+      <c r="G643" s="15" t="s">
         <v>1171</v>
       </c>
       <c r="H643" s="10" t="s">
@@ -19950,7 +19949,7 @@
       <c r="E650" s="9" t="s">
         <v>1181</v>
       </c>
-      <c r="G650" s="16" t="s">
+      <c r="G650" s="15" t="s">
         <v>1182</v>
       </c>
       <c r="H650" s="10" t="s">
@@ -20038,7 +20037,7 @@
       <c r="E655" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="G655" s="16" t="s">
+      <c r="G655" s="15" t="s">
         <v>1189</v>
       </c>
       <c r="H655" s="10" t="s">
@@ -24455,7 +24454,7 @@
         <v>6167</v>
       </c>
       <c r="D923" s="9" t="s">
-        <v>1636</v>
+        <v>1632</v>
       </c>
       <c r="E923" s="9" t="s">
         <v>1637</v>
@@ -24557,7 +24556,7 @@
         <v>6254</v>
       </c>
       <c r="D929" s="9" t="s">
-        <v>1636</v>
+        <v>1632</v>
       </c>
       <c r="E929" s="9" t="s">
         <v>119</v>
@@ -25637,7 +25636,7 @@
       <c r="F994" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="G994" s="16" t="s">
+      <c r="G994" s="15" t="s">
         <v>1779</v>
       </c>
       <c r="H994" s="10" t="s">
@@ -25654,7 +25653,7 @@
       <c r="F995" s="9" t="s">
         <v>1781</v>
       </c>
-      <c r="G995" s="16" t="s">
+      <c r="G995" s="15" t="s">
         <v>1782</v>
       </c>
       <c r="H995" s="10" t="s">
@@ -25713,7 +25712,7 @@
       <c r="F999" s="9" t="s">
         <v>1785</v>
       </c>
-      <c r="G999" s="16" t="s">
+      <c r="G999" s="15" t="s">
         <v>1786</v>
       </c>
       <c r="H999" s="10" t="s">
@@ -25730,7 +25729,7 @@
       <c r="F1000" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="G1000" s="16" t="s">
+      <c r="G1000" s="15" t="s">
         <v>1788</v>
       </c>
     </row>
@@ -25744,7 +25743,7 @@
       <c r="F1001" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="G1001" s="16" t="s">
+      <c r="G1001" s="15" t="s">
         <v>1789</v>
       </c>
       <c r="H1001" s="10" t="s">
@@ -25899,7 +25898,7 @@
       <c r="A1011" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B1011" s="17">
+      <c r="B1011" s="16">
         <v>6854.2</v>
       </c>
       <c r="F1011" s="9" t="s">
@@ -25916,7 +25915,7 @@
       <c r="A1012" s="9" t="s">
         <v>2120</v>
       </c>
-      <c r="B1012" s="17">
+      <c r="B1012" s="16">
         <v>6859</v>
       </c>
       <c r="F1012" s="9" t="s">
@@ -29124,7 +29123,7 @@
       <c r="A1212" s="9" t="s">
         <v>2120</v>
       </c>
-      <c r="B1212" s="17">
+      <c r="B1212" s="16">
         <v>8158.2</v>
       </c>
       <c r="F1212" s="9" t="s">

</xml_diff>

<commit_message>
corr(data): resolve ambiguous naming attributions across the corpus
Nine rows carried both 'Nennende Figur' and 'Erzähler', two Iwein rows
carried neither. Every naming row now holds exactly one attribution:
figure speech, narrator or self-naming.

- Rolandslied: 8 rows (V. 527, 2863, 2864, 2875, 2880, 2882, 2887, 6101)
- Iwein: 3 rows (V. 1805, 2216, 4905)
- Trojanerkrieg: 2 rows (V. 4272, 36644; the latter a spelling fix)

The corrections were carried into the 'Gesamt' and 'lemmatisiert' sheets
of the export workbooks. These were edited on package level so that cell
comments and table definitions survive unchanged.
</commit_message>
<xml_diff>
--- a/data/Iwein/Iwein_final.xlsx
+++ b/data/Iwein/Iwein_final.xlsx
@@ -5914,14 +5914,15 @@
       </c>
       <c r="D205" s="9" t="inlineStr">
         <is>
-          <t>Lunete</t>
-        </is>
-      </c>
-      <c r="F205" s="9" t="inlineStr">
-        <is>
-          <t>vrouwe</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Lunete</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vrouwe</t>
+        </is>
+      </c>
+      <c r="F205" s="9"/>
       <c r="G205" s="9" t="inlineStr">
         <is>
           <t>›meinstûz sô?‹ ›vrouwe, jâ.‹</t>
@@ -7753,9 +7754,10 @@
       <c r="B276" s="9" t="n">
         <v>2216</v>
       </c>
-      <c r="E276" s="9" t="inlineStr">
-        <is>
-          <t>iunchvrouwe</t>
+      <c r="E276" s="9"/>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">iunchvrouwe</t>
         </is>
       </c>
       <c r="G276" s="9" t="inlineStr">
@@ -17721,9 +17723,14 @@
       <c r="B676" s="9" t="n">
         <v>4905</v>
       </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Iwein</t>
+        </is>
+      </c>
       <c r="E676" s="9" t="inlineStr">
         <is>
-          <t>hern Gâweins</t>
+          <t xml:space="preserve">hern Gâweins</t>
         </is>
       </c>
       <c r="G676" s="9" t="inlineStr">
@@ -39939,13 +39946,13 @@
         <v>2216</v>
       </c>
       <c r="C269" s="2" t="n"/>
-      <c r="D269" s="2" t="n"/>
-      <c r="E269" s="2" t="inlineStr">
-        <is>
-          <t>iunchvrouwe</t>
-        </is>
-      </c>
-      <c r="F269" s="2" t="n"/>
+      <c r="D269" s="2"/>
+      <c r="E269" s="2"/>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">iunchvrouwe</t>
+        </is>
+      </c>
       <c r="G269" s="2" t="inlineStr">
         <is>
           <t>juncvrouwe</t>
@@ -53338,13 +53345,17 @@
         <v>4905</v>
       </c>
       <c r="C655" s="2" t="n"/>
-      <c r="D655" s="2" t="n"/>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Iwein</t>
+        </is>
+      </c>
       <c r="E655" s="2" t="inlineStr">
         <is>
-          <t>hern Gâweins</t>
-        </is>
-      </c>
-      <c r="F655" s="2" t="n"/>
+          <t xml:space="preserve">hern Gâweins</t>
+        </is>
+      </c>
+      <c r="F655" s="2"/>
       <c r="G655" s="2" t="inlineStr">
         <is>
           <t>hêrre</t>

</xml_diff>